<commit_message>
Notação: som de law/thought/chocolate passa a ser 'á' (Cambridge US)
- 26 palavras ajustadas (chocolate, thought, talk, walk, because...) e pares mínimos
- Legenda: 'ó' só antes de R; nova linha para o i átono no fim (city SI-ɾi)
- validar.py acusa 'ó' sem R depois
- cambridge.py: consulta o IPA US e confere a planilha inteira

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ULtze7ZBLf8ZSPzUELZjA5
</commit_message>
<xml_diff>
--- a/Guia_Ingles_Pronuncia.xlsx
+++ b/Guia_Ingles_Pronuncia.xlsx
@@ -1151,7 +1151,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1272,415 +1272,419 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>é</t>
+          <t>i (átono no fim)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>ɛ</t>
+          <t>i</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>É de "pé"</t>
+          <t>No fim da palavra, sem acento, o i é curto e leve, mesmo quando o IPA mostra /i/</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>bed = BÉD · men = MÉN</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
+          <t>city = SI-ɾi · family = FÆM-li</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Alongar: "sitii", "fæmilii"</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>æ</t>
+          <t>é</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>æ</t>
+          <t>ɛ</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Boca aberta como para "á", mas falando "é"</t>
+          <t>É de "pé"</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>bad = BÆD · man = MÆN</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Falar "é" de pé: bad vira bed</t>
-        </is>
-      </c>
+          <t>bed = BÉD · men = MÉN</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>á</t>
+          <t>æ</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>ɑ</t>
+          <t>æ</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Á com a boca bem aberta, som do fundo</t>
+          <t>Boca aberta como para "á", mas falando "é"</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>hot = HÁT · doctor = DÁK-târ</t>
+          <t>bad = BÆD · man = MÆN</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Falar "ó" (é britânico, não americano)</t>
+          <t>Falar "é" de pé: bad vira bed</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ó</t>
+          <t>á</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>ɔ</t>
+          <t>ɑ</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Ó de "avó". Muitos americanos falam "á": os dois são aceitos</t>
+          <t>Á com a boca bem aberta, som do fundo. Vale para hot e doctor e também para law, thought, talk, walk e because</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>law = LÓ · thought = THÓT</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
+          <t>hot = HÁT · law = LÁ · walk = WÁK</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Falar "ó" (é britânico, não americano)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>â / Â</t>
+          <t>ór</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>ə / ʌ</t>
+          <t>ɔr</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Â de "cama", curto e solto. Átono (minúsculo) é quase murmurado</t>
+          <t>Ó de "avó", só antes de R. Sem R, o guia usa á (Cambridge US); muitos americanos do Leste falam "ó", também aceito</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>about = â-BÁUT · cup = KÂP</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Ler a vogal escrita: "abáut", "cúp"</t>
-        </is>
-      </c>
+          <t>more = MÓR · four = FÓR</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>u</t>
+          <t>â / Â</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>ʊ</t>
+          <t>ə / ʌ</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>U curto e relaxado, quase "ô"</t>
+          <t>Â de "cama", curto e solto. Átono (minúsculo) é quase murmurado</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>book = BUK · good = GUD</t>
+          <t>about = â-BÁUT · cup = KÂP</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Falar o "u" longo: full vira fool</t>
+          <t>Ler a vogal escrita: "abáut", "cúp"</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>uu</t>
+          <t>u</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>u</t>
+          <t>ʊ</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>U longo, com os lábios em bico</t>
+          <t>U curto e relaxado, quase "ô"</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>food = FUUD · two = TUU</t>
+          <t>book = BUK · good = GUD</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Encurtar: pool vira pull</t>
+          <t>Falar o "u" longo: full vira fool</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>âr</t>
+          <t>uu</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>ɚ / ɝ</t>
+          <t>u</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Â seguido de R americano, quase uma vogal só</t>
+          <t>U longo, com os lábios em bico</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>work = WÂRK · teacher = TII-tchâr</t>
+          <t>food = FUUD · two = TUU</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Falar "ór" ou "ér": work vira walk</t>
+          <t>Encurtar: pool vira pull</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>êi · ôu · ái · áu · ói</t>
+          <t>âr</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>eɪ oʊ aɪ aʊ ɔɪ</t>
+          <t>ɚ / ɝ</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Ditongos: as duas vogais soam</t>
+          <t>Â seguido de R americano, quase uma vogal só</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>day = DÊI · go = GÔU · night = NÁIT</t>
+          <t>work = WÂRK · teacher = TII-tchâr</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Cortar o ditongo: "gô" em vez de GÔU</t>
+          <t>Falar "ór" ou "ér": work vira walk</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>r</t>
+          <t>êi · ôu · ái · áu · ói</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>ɹ</t>
+          <t>eɪ oʊ aɪ aʊ ɔɪ</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>R americano: língua curvada para trás, sem encostar e sem vibrar</t>
+          <t>Ditongos: as duas vogais soam</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>red = RÉD · car = KÁR</t>
+          <t>day = DÊI · go = GÔU · night = NÁIT</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Usar o R de "rato": em inglês ele soa como H (red vira head)</t>
+          <t>Cortar o ditongo: "gô" em vez de GÔU</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>ɾ</t>
+          <t>r</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>ɾ</t>
+          <t>ɹ</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Toque rápido de língua, como o r de "caro". É o T ou D entre vogais</t>
+          <t>R americano: língua curvada para trás, sem encostar e sem vibrar</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>better = BÉ-ɾâr · city = SI-ɾi</t>
+          <t>red = RÉD · car = KÁR</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Falar T cheio ("bé-ter") ou "tchi"</t>
+          <t>Usar o R de "rato": em inglês ele soa como H (red vira head)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>t'</t>
+          <t>ɾ</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>ʔ</t>
+          <t>ɾ</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>T preso na garganta, sem soltar ar, antes de N</t>
+          <t>Toque rápido de língua, como o r de "caro". É o T ou D entre vogais</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>button = BÂ-t'n</t>
+          <t>better = BÉ-ɾâr · city = SI-ɾi</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Falar "bâ-tôn" com vogal</t>
+          <t>Falar T cheio ("bé-ter") ou "tchi"</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>th</t>
+          <t>t'</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>θ</t>
+          <t>ʔ</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Língua entre os dentes, sopro sem voz</t>
+          <t>T preso na garganta, sem soltar ar, antes de N</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>think = THINK</t>
+          <t>button = BÂ-t'n</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Trocar por T, F ou S: "tink", "fink"</t>
+          <t>Falar "bâ-tôn" com vogal</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>dh</t>
+          <t>th</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>ð</t>
+          <t>θ</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Igual ao th, mas com voz (vibra)</t>
+          <t>Língua entre os dentes, sopro sem voz</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>this = DHIS · mother = MÂ-dhâr</t>
+          <t>think = THINK</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Trocar por D: "dis"</t>
+          <t>Trocar por T, F ou S: "tink", "fink"</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>h</t>
+          <t>dh</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>h</t>
+          <t>ð</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Sopro, como o R de "rato" no Rio</t>
+          <t>Igual ao th, mas com voz (vibra)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>house = HÁUS · hot = HÁT</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr"/>
+          <t>this = DHIS · mother = MÂ-dhâr</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Trocar por D: "dis"</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>sh · tch</t>
+          <t>h</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>ʃ · tʃ</t>
+          <t>h</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>"ch" de chuva · "tch" de tchau</t>
+          <t>Sopro, como o R de "rato" no Rio</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>she = SHII · church = TCHÂRTCH</t>
+          <t>house = HÁUS · hot = HÁT</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
@@ -1688,156 +1692,179 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>j · dj</t>
+          <t>sh · tch</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>ʒ · dʒ</t>
+          <t>ʃ · tʃ</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>"j" de já · "dj" de adjetivo</t>
+          <t>"ch" de chuva · "tch" de tchau</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>measure = MÉ-jâr · job = DJÁB</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Trocar um pelo outro</t>
-        </is>
-      </c>
+          <t>she = SHII · church = TCHÂRTCH</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>w · y</t>
+          <t>j · dj</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>w · j</t>
+          <t>ʒ · dʒ</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>"u" rápido (como em quase) · "i" rápido (como em iate)</t>
+          <t>"j" de já · "dj" de adjetivo</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>walk = WÓK · yes = YÉS</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr"/>
+          <t>measure = MÉ-jâr · job = DJÁB</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Trocar um pelo outro</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>w · y</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>w · j</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Ponta da língua toca a gengiva atrás dos dentes de cima</t>
+          <t>"u" rápido (como em quase) · "i" rápido (como em iate)</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>nation = NÊI-shân · sin = SIN</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>Terminar em vogal nasal ("xã") sem fechar</t>
-        </is>
-      </c>
+          <t>walk = WÁK · yes = YÉS</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>ng</t>
+          <t>n</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>ŋ</t>
+          <t>n</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Fundo da língua sobe até o céu da boca; não solte o G</t>
+          <t>Ponta da língua toca a gengiva atrás dos dentes de cima</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>sing = SING · working = WÂR-king</t>
+          <t>nation = NÊI-shân · sin = SIN</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>"sin-gui" (soltando o G) ou só vogal nasal</t>
+          <t>Terminar em vogal nasal ("xã") sem fechar</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ng</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ŋ</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Lábios fechados de verdade</t>
+          <t>Fundo da língua sobe até o céu da boca; não solte o G</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>problem = PRÁ-blâm · sum = SÂM</t>
+          <t>sing = SING · working = WÂR-king</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>"probleim" (vogal nasal, sem fechar os lábios)</t>
+          <t>"sin-gui" (soltando o G) ou só vogal nasal</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Lábios fechados de verdade</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>problem = PRÁ-blâm · sum = SÂM</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>"probleim" (vogal nasal, sem fechar os lábios)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
           <t>l (fim de sílaba)</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>ɫ</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>L escuro: a ponta da língua toca atrás dos dentes. Não vira "u"</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>feel = FIIL · people = PII-pâl</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>"fiu", "pípou" (L virando U, como em Brasil)</t>
         </is>
@@ -2178,7 +2205,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>É a mesma regra do -S: o som anterior decide. Cuidado com walked (WÓKT) × worked (WÂRKT): é o par walk/work.</t>
+          <t>É a mesma regra do -S: o som anterior decide. Cuidado com walked (WÁKT) × worked (WÂRKT): é o par walk/work.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -2648,7 +2675,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Átono. Mesmo L escuro em all (ÓL), tell (TÉL), feel (FIIL), call (KÓL).</t>
+          <t>Átono. Mesmo L escuro em all (ÁL), tell (TÉL), feel (FIIL), call (KÁL).</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -3212,7 +3239,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>O acento nunca cai no -ity. Mesmo ɾ em city (SI-ɾi), party (PÁR-ɾi), better (BÉ-ɾâr), water (WÓ-ɾâr).</t>
+          <t>O acento nunca cai no -ity. Mesmo ɾ em city (SI-ɾi), party (PÁR-ɾi), better (BÉ-ɾâr), water (WÁ-ɾâr).</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -3437,7 +3464,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>ó</t>
+          <t>á</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -3447,7 +3474,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Mesmo som em -AW: law (LÓ), saw (SÓ), draw (DRÓ). Muitos americanos falam "á" (LÁ): os dois são aceitos. Exceções: laugh (LÆF), aunt (ÆNT).</t>
+          <t>Mesmo som em -AW: law (LÁ), saw (SÁ), draw (DRÁ). Também se ouve "ó" (LÓ), mais no Leste dos EUA: os dois são aceitos; o guia segue o Cambridge US (á). Exceções: laugh (LÆF), aunt (ÆNT).</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3531,17 +3558,17 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>ót</t>
+          <t>át</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Ler "ou" como "ou" ou "af". Os dois finais têm o mesmo "ót" (AU = ó).</t>
+          <t>Ler "ou" como "ou" ou "af". Os dois finais têm o mesmo "át" (AU = á).</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Também: daughter (DÓ-ɾâr), naughty (NÓ-ɾi).</t>
+          <t>Também: daughter (DÁ-ɾâr), naughty (NÁ-ɾi).</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -3578,7 +3605,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>varia: ôu, uu, âf, óf, áu</t>
+          <t>varia: ôu, uu, âf, áf, áu</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -3776,7 +3803,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Em often, o T é opcional (Ó-fân é o mais comum). Em tsunami, "suu-NÁ-mi" e "tsuu-NÁ-mi" são aceitos.</t>
+          <t>Em often, o T é opcional (Á-fân é o mais comum). Em tsunami, "suu-NÁ-mi" e "tsuu-NÁ-mi" são aceitos.</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -4832,12 +4859,12 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>WÓKT</t>
+          <t>WÁKT</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>wɔkt</t>
+          <t>wɑkt</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -5054,12 +5081,12 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>KÓLD</t>
+          <t>KÁLD</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>kɔld</t>
+          <t>kɑld</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -6977,12 +7004,12 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>KÓL</t>
+          <t>KÁL</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>kɔl</t>
+          <t>kɑl</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
@@ -9715,12 +9742,12 @@
       </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>TCHÓK-lât</t>
+          <t>TCHÁK-lât</t>
         </is>
       </c>
       <c r="E151" s="2" t="inlineStr">
         <is>
-          <t>ˈtʃɔklət</t>
+          <t>ˈtʃɑklət</t>
         </is>
       </c>
       <c r="F151" s="2" t="inlineStr">
@@ -11774,12 +11801,12 @@
       </c>
       <c r="D210" s="2" t="inlineStr">
         <is>
-          <t>bi-KÓZ</t>
+          <t>bi-KÁZ</t>
         </is>
       </c>
       <c r="E210" s="2" t="inlineStr">
         <is>
-          <t>bɪˈkɔz</t>
+          <t>bɪˈkɑz</t>
         </is>
       </c>
       <c r="F210" s="2" t="inlineStr">
@@ -11807,12 +11834,12 @@
       </c>
       <c r="D211" s="2" t="inlineStr">
         <is>
-          <t>Ó-thâr</t>
+          <t>Á-thâr</t>
         </is>
       </c>
       <c r="E211" s="2" t="inlineStr">
         <is>
-          <t>ˈɔθɚ</t>
+          <t>ˈɑθɚ</t>
         </is>
       </c>
       <c r="F211" s="2" t="inlineStr">
@@ -11840,12 +11867,12 @@
       </c>
       <c r="D212" s="2" t="inlineStr">
         <is>
-          <t>Ó-gâst</t>
+          <t>Á-gâst</t>
         </is>
       </c>
       <c r="E212" s="2" t="inlineStr">
         <is>
-          <t>ˈɔɡəst</t>
+          <t>ˈɑɡəst</t>
         </is>
       </c>
       <c r="F212" s="2" t="inlineStr">
@@ -11873,12 +11900,12 @@
       </c>
       <c r="D213" s="2" t="inlineStr">
         <is>
-          <t>PÓZ</t>
+          <t>PÁZ</t>
         </is>
       </c>
       <c r="E213" s="2" t="inlineStr">
         <is>
-          <t>pɔz</t>
+          <t>pɑz</t>
         </is>
       </c>
       <c r="F213" s="2" t="inlineStr">
@@ -11906,12 +11933,12 @@
       </c>
       <c r="D214" s="2" t="inlineStr">
         <is>
-          <t>SÓS</t>
+          <t>SÁS</t>
         </is>
       </c>
       <c r="E214" s="2" t="inlineStr">
         <is>
-          <t>sɔs</t>
+          <t>sɑs</t>
         </is>
       </c>
       <c r="F214" s="2" t="inlineStr">
@@ -11939,12 +11966,12 @@
       </c>
       <c r="D215" s="2" t="inlineStr">
         <is>
-          <t>FÓLT</t>
+          <t>FÁLT</t>
         </is>
       </c>
       <c r="E215" s="2" t="inlineStr">
         <is>
-          <t>fɔlt</t>
+          <t>fɑlt</t>
         </is>
       </c>
       <c r="F215" s="2" t="inlineStr">
@@ -11972,12 +11999,12 @@
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>ó-ɾâ-MÆ-ɾik</t>
+          <t>á-ɾâ-MÆ-ɾik</t>
         </is>
       </c>
       <c r="E216" s="2" t="inlineStr">
         <is>
-          <t>ˌɔɾəˈmæɾɪk</t>
+          <t>ˌɑɾəˈmæɾɪk</t>
         </is>
       </c>
       <c r="F216" s="2" t="inlineStr">
@@ -12005,12 +12032,12 @@
       </c>
       <c r="D217" s="2" t="inlineStr">
         <is>
-          <t>Ó-ɾâm</t>
+          <t>Á-ɾâm</t>
         </is>
       </c>
       <c r="E217" s="2" t="inlineStr">
         <is>
-          <t>ˈɔɾəm</t>
+          <t>ˈɑɾəm</t>
         </is>
       </c>
       <c r="F217" s="2" t="inlineStr">
@@ -12038,12 +12065,12 @@
       </c>
       <c r="D218" s="2" t="inlineStr">
         <is>
-          <t>LÓN-dri</t>
+          <t>LÁN-dri</t>
         </is>
       </c>
       <c r="E218" s="2" t="inlineStr">
         <is>
-          <t>ˈlɔndri</t>
+          <t>ˈlɑndri</t>
         </is>
       </c>
       <c r="F218" s="2" t="inlineStr">
@@ -12269,12 +12296,12 @@
       </c>
       <c r="D225" s="2" t="inlineStr">
         <is>
-          <t>THÓT</t>
+          <t>THÁT</t>
         </is>
       </c>
       <c r="E225" s="2" t="inlineStr">
         <is>
-          <t>θɔt</t>
+          <t>θɑt</t>
         </is>
       </c>
       <c r="F225" s="2" t="inlineStr">
@@ -12302,12 +12329,12 @@
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>BÓT</t>
+          <t>BÁT</t>
         </is>
       </c>
       <c r="E226" s="2" t="inlineStr">
         <is>
-          <t>bɔt</t>
+          <t>bɑt</t>
         </is>
       </c>
       <c r="F226" s="2" t="inlineStr">
@@ -12335,12 +12362,12 @@
       </c>
       <c r="D227" s="2" t="inlineStr">
         <is>
-          <t>BRÓT</t>
+          <t>BRÁT</t>
         </is>
       </c>
       <c r="E227" s="2" t="inlineStr">
         <is>
-          <t>brɔt</t>
+          <t>brɑt</t>
         </is>
       </c>
       <c r="F227" s="2" t="inlineStr">
@@ -12368,12 +12395,12 @@
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t>KÓT</t>
+          <t>KÁT</t>
         </is>
       </c>
       <c r="E228" s="2" t="inlineStr">
         <is>
-          <t>kɔt</t>
+          <t>kɑt</t>
         </is>
       </c>
       <c r="F228" s="2" t="inlineStr">
@@ -12401,12 +12428,12 @@
       </c>
       <c r="D229" s="2" t="inlineStr">
         <is>
-          <t>TÓT</t>
+          <t>TÁT</t>
         </is>
       </c>
       <c r="E229" s="2" t="inlineStr">
         <is>
-          <t>tɔt</t>
+          <t>tɑt</t>
         </is>
       </c>
       <c r="F229" s="2" t="inlineStr">
@@ -12434,12 +12461,12 @@
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>FÓT</t>
+          <t>FÁT</t>
         </is>
       </c>
       <c r="E230" s="2" t="inlineStr">
         <is>
-          <t>fɔt</t>
+          <t>fɑt</t>
         </is>
       </c>
       <c r="F230" s="2" t="inlineStr">
@@ -12508,12 +12535,12 @@
       </c>
       <c r="D232" s="2" t="inlineStr">
         <is>
-          <t>ól-DHÔU</t>
+          <t>ál-DHÔU</t>
         </is>
       </c>
       <c r="E232" s="2" t="inlineStr">
         <is>
-          <t>ɔlˈðoʊ</t>
+          <t>ɑlˈðoʊ</t>
         </is>
       </c>
       <c r="F232" s="2" t="inlineStr">
@@ -12720,7 +12747,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>óf</t>
+          <t>áf</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -12730,12 +12757,12 @@
       </c>
       <c r="D238" s="2" t="inlineStr">
         <is>
-          <t>KÓF</t>
+          <t>KÁF</t>
         </is>
       </c>
       <c r="E238" s="2" t="inlineStr">
         <is>
-          <t>kɔf</t>
+          <t>kɑf</t>
         </is>
       </c>
       <c r="F238" s="2" t="inlineStr">
@@ -13763,12 +13790,12 @@
       </c>
       <c r="D267" s="2" t="inlineStr">
         <is>
-          <t>Ó-fân</t>
+          <t>Á-fân</t>
         </is>
       </c>
       <c r="E267" s="2" t="inlineStr">
         <is>
-          <t>ˈɔfən</t>
+          <t>ˈɑfən</t>
         </is>
       </c>
       <c r="F267" s="2" t="inlineStr">
@@ -14720,12 +14747,12 @@
       </c>
       <c r="D296" s="2" t="inlineStr">
         <is>
-          <t>RÓNG</t>
+          <t>RÁNG</t>
         </is>
       </c>
       <c r="E296" s="2" t="inlineStr">
         <is>
-          <t>rɔŋ</t>
+          <t>rɑŋ</t>
         </is>
       </c>
       <c r="F296" s="2" t="inlineStr">
@@ -15149,12 +15176,12 @@
       </c>
       <c r="D309" s="2" t="inlineStr">
         <is>
-          <t>TÓK</t>
+          <t>TÁK</t>
         </is>
       </c>
       <c r="E309" s="2" t="inlineStr">
         <is>
-          <t>tɔk</t>
+          <t>tɑk</t>
         </is>
       </c>
       <c r="F309" s="2" t="inlineStr">
@@ -15182,12 +15209,12 @@
       </c>
       <c r="D310" s="2" t="inlineStr">
         <is>
-          <t>WÓK</t>
+          <t>WÁK</t>
         </is>
       </c>
       <c r="E310" s="2" t="inlineStr">
         <is>
-          <t>wɔk</t>
+          <t>wɑk</t>
         </is>
       </c>
       <c r="F310" s="2" t="inlineStr">
@@ -15941,12 +15968,12 @@
       </c>
       <c r="D333" s="2" t="inlineStr">
         <is>
-          <t>DÓ-ɾâr</t>
+          <t>DÁ-ɾâr</t>
         </is>
       </c>
       <c r="E333" s="2" t="inlineStr">
         <is>
-          <t>ˈdɔɾɚ</t>
+          <t>ˈdɑɾɚ</t>
         </is>
       </c>
       <c r="F333" s="2" t="inlineStr">
@@ -18406,7 +18433,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>âr × ór</t>
+          <t>âr × á / ór</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -18426,7 +18453,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>WÓK</t>
+          <t>WÁK</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr"/>
@@ -18435,7 +18462,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>âr × ór</t>
+          <t>âr × á / ór</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -18455,7 +18482,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>WÓKT</t>
+          <t>WÁKT</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr"/>
@@ -18464,7 +18491,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>âr × ór</t>
+          <t>âr × á / ór</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -18493,7 +18520,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>âr × ór</t>
+          <t>âr × á / ór</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -18627,7 +18654,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>THÓT</t>
+          <t>THÁT</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -18637,7 +18664,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>TÓT</t>
+          <t>TÁT</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr"/>
@@ -18853,12 +18880,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>âr × ór</t>
+          <t>âr × á / ór</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>âr (work, bird) × ór (walk, board). Confundir troca a palavra.</t>
+          <t>âr (work, bird, shirt) × á (walk) e ór (board, short). Confundir troca a palavra.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inclui post @ingles.doimigrante e ampliação: seção Fala do dia a dia e 83 palavras
- Nova seção Fala do dia a dia: reduções (gonna, wanna...), T/D + YOU, formas fracas, conectores
- Novos grupos: E final que soa (recipe...), Grafia que engana (clothes, colonel, women...)
- mortgage em T mudo; pares mínimos can × can't e recipe × receipt
- magazine = mæ-gâ-ZIIN (Cambridge US)
- cambridge.py trata ər/ɜr como ɚ/ɝ na comparação

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ULtze7ZBLf8ZSPzUELZjA5
</commit_message>
<xml_diff>
--- a/Guia_Ingles_Pronuncia.xlsx
+++ b/Guia_Ingles_Pronuncia.xlsx
@@ -1882,7 +1882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2054,6 +2054,21 @@
       <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Palavras de reunião, projeto e fábrica que costumam sair erradas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Fala do dia a dia</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Como os americanos falam de verdade: reduções, palavras que se juntam, formas fracas e conectores.</t>
         </is>
       </c>
     </row>
@@ -2069,7 +2084,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4571,6 +4586,288 @@
       <c r="I53" s="2" t="inlineStr">
         <is>
           <t>Revisão out/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Fala do dia a dia</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Reduções informais</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>TO, OF e HAVE viram â</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Usar gonna para movimento ("I'm gonna the store") ou escrever gonna e wanna em e-mail de trabalho.</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Gonna só no futuro (going to + verbo). Com he/she, wanna vira wants to (WÁNTS-tâ). É fala informal: na escrita formal, use a forma completa.</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>I'm gonna call you later, I gotta go. Lemme see... I dunno.</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>JUNC</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Fala do dia a dia</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>T/D + YOU</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>t + y = tch | d + y = dj</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Separar as palavras: "dont iu", "did iu", "uót ar iu".</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Acontece em toda junção de T ou D com Y, mesmo sem "you": last year (læs-TCHIR).</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Whatcha doing? Didja get my message? Gotcha, nice to meet you.</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>FRACAS</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Fala do dia a dia</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Formas fracas</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>â no lugar da vogal cheia</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Pronunciar cada palavrinha com a vogal cheia: "tuu", "fór", "ænd", "yuu". A fala fica robótica.</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>A forma forte (entre parênteses) só aparece com ênfase ou no fim da frase: Who is it for? (FÓR). O H de him/her some no meio da frase: tell him = TÉ-lim.</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>I have to go to work for an hour and call them at ten.</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>CONECT</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Fala do dia a dia</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Conectores</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>tônica e ditongos que somem</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>"bé-cá-uze" com áu, "rau-éver", "éni-uêi", "ól-so" com o fechado.</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Na fala rápida, because vira 'cause (KÂZ) e but perde o T final (BÂ'). Use anyway, não anyways, em contexto formal.</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Anyway, the pump is fine. However, we should check the valve instead, because it leaks.</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>EFINAL</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Vogais com grafia traiçoeira</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>E final que soa</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>i (o E final é sílaba)</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Ler o E final como mudo: "re-SÁIP", "kâ-RÊIT", "ékn".</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Quase sempre palavras de origem grega, latina, espanhola ou japonesa. Recipe ≠ receipt: RÉ-sâ-pi (receita) × ri-SIIT (recibo).</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>The recipe for the karate team's sesame cake was a catastrophe.</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>Pontual</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>GRAF</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Vogais com grafia traiçoeira</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Grafia que engana</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>sem regra: decorar uma a uma</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Ler pela escrita: "côlonel", "uómen", "biúzi", "clôu-zis", "fébruári".</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Women: o O soa como i curto (WI-min); woman, no singular, é WU-mân. Clothes: o TH quase some na fala (KLÔUZ).</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>The colonel says the women are pretty busy this February.</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
         </is>
       </c>
     </row>
@@ -4594,7 +4891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G386"/>
+  <dimension ref="A1:G469"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -17731,6 +18028,2933 @@
         </is>
       </c>
       <c r="G386" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="2" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="B387" s="2" t="inlineStr">
+        <is>
+          <t>TO vira tâ</t>
+        </is>
+      </c>
+      <c r="C387" s="2" t="inlineStr">
+        <is>
+          <t>gonna (going to)</t>
+        </is>
+      </c>
+      <c r="D387" s="2" t="inlineStr">
+        <is>
+          <t>GÁ-nâ</t>
+        </is>
+      </c>
+      <c r="E387" s="2" t="inlineStr">
+        <is>
+          <t>ˈɡɑnə</t>
+        </is>
+      </c>
+      <c r="F387" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+      <c r="G387" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="2" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="B388" s="2" t="inlineStr">
+        <is>
+          <t>TO vira tâ</t>
+        </is>
+      </c>
+      <c r="C388" s="2" t="inlineStr">
+        <is>
+          <t>wanna (want to)</t>
+        </is>
+      </c>
+      <c r="D388" s="2" t="inlineStr">
+        <is>
+          <t>WÁ-nâ</t>
+        </is>
+      </c>
+      <c r="E388" s="2" t="inlineStr">
+        <is>
+          <t>ˈwɑnə</t>
+        </is>
+      </c>
+      <c r="F388" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+      <c r="G388" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="2" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="B389" s="2" t="inlineStr">
+        <is>
+          <t>TO vira tâ</t>
+        </is>
+      </c>
+      <c r="C389" s="2" t="inlineStr">
+        <is>
+          <t>gotta (got to)</t>
+        </is>
+      </c>
+      <c r="D389" s="2" t="inlineStr">
+        <is>
+          <t>GÁ-ɾâ</t>
+        </is>
+      </c>
+      <c r="E389" s="2" t="inlineStr">
+        <is>
+          <t>ˈɡɑɾə</t>
+        </is>
+      </c>
+      <c r="F389" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+      <c r="G389" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="2" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="B390" s="2" t="inlineStr">
+        <is>
+          <t>TO vira tâ</t>
+        </is>
+      </c>
+      <c r="C390" s="2" t="inlineStr">
+        <is>
+          <t>hafta (have to)</t>
+        </is>
+      </c>
+      <c r="D390" s="2" t="inlineStr">
+        <is>
+          <t>HÆF-tâ</t>
+        </is>
+      </c>
+      <c r="E390" s="2" t="inlineStr">
+        <is>
+          <t>ˈhæftə</t>
+        </is>
+      </c>
+      <c r="F390" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+      <c r="G390" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="2" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="B391" s="2" t="inlineStr">
+        <is>
+          <t>TO vira tâ</t>
+        </is>
+      </c>
+      <c r="C391" s="2" t="inlineStr">
+        <is>
+          <t>hasta (has to)</t>
+        </is>
+      </c>
+      <c r="D391" s="2" t="inlineStr">
+        <is>
+          <t>HÆS-tâ</t>
+        </is>
+      </c>
+      <c r="E391" s="2" t="inlineStr">
+        <is>
+          <t>ˈhæstə</t>
+        </is>
+      </c>
+      <c r="F391" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G391" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="2" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="B392" s="2" t="inlineStr">
+        <is>
+          <t>TO vira tâ</t>
+        </is>
+      </c>
+      <c r="C392" s="2" t="inlineStr">
+        <is>
+          <t>usta (used to)</t>
+        </is>
+      </c>
+      <c r="D392" s="2" t="inlineStr">
+        <is>
+          <t>YUUS-tâ</t>
+        </is>
+      </c>
+      <c r="E392" s="2" t="inlineStr">
+        <is>
+          <t>ˈjustə</t>
+        </is>
+      </c>
+      <c r="F392" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G392" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="2" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="B393" s="2" t="inlineStr">
+        <is>
+          <t>TO vira tâ</t>
+        </is>
+      </c>
+      <c r="C393" s="2" t="inlineStr">
+        <is>
+          <t>supposta (supposed to)</t>
+        </is>
+      </c>
+      <c r="D393" s="2" t="inlineStr">
+        <is>
+          <t>sâ-PÔUS-tâ</t>
+        </is>
+      </c>
+      <c r="E393" s="2" t="inlineStr">
+        <is>
+          <t>səˈpoʊstə</t>
+        </is>
+      </c>
+      <c r="F393" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G393" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="2" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="B394" s="2" t="inlineStr">
+        <is>
+          <t>TO vira tâ</t>
+        </is>
+      </c>
+      <c r="C394" s="2" t="inlineStr">
+        <is>
+          <t>tryna (trying to)</t>
+        </is>
+      </c>
+      <c r="D394" s="2" t="inlineStr">
+        <is>
+          <t>TRÁI-nâ</t>
+        </is>
+      </c>
+      <c r="E394" s="2" t="inlineStr">
+        <is>
+          <t>ˈtraɪnə</t>
+        </is>
+      </c>
+      <c r="F394" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G394" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="2" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="B395" s="2" t="inlineStr">
+        <is>
+          <t>OF vira â</t>
+        </is>
+      </c>
+      <c r="C395" s="2" t="inlineStr">
+        <is>
+          <t>kinda (kind of)</t>
+        </is>
+      </c>
+      <c r="D395" s="2" t="inlineStr">
+        <is>
+          <t>KÁIN-dâ</t>
+        </is>
+      </c>
+      <c r="E395" s="2" t="inlineStr">
+        <is>
+          <t>ˈkaɪndə</t>
+        </is>
+      </c>
+      <c r="F395" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+      <c r="G395" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="2" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="B396" s="2" t="inlineStr">
+        <is>
+          <t>OF vira â</t>
+        </is>
+      </c>
+      <c r="C396" s="2" t="inlineStr">
+        <is>
+          <t>sorta (sort of)</t>
+        </is>
+      </c>
+      <c r="D396" s="2" t="inlineStr">
+        <is>
+          <t>SÓR-ɾâ</t>
+        </is>
+      </c>
+      <c r="E396" s="2" t="inlineStr">
+        <is>
+          <t>ˈsɔrɾə</t>
+        </is>
+      </c>
+      <c r="F396" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G396" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="2" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="B397" s="2" t="inlineStr">
+        <is>
+          <t>OF vira â</t>
+        </is>
+      </c>
+      <c r="C397" s="2" t="inlineStr">
+        <is>
+          <t>outta (out of)</t>
+        </is>
+      </c>
+      <c r="D397" s="2" t="inlineStr">
+        <is>
+          <t>ÁU-ɾâ</t>
+        </is>
+      </c>
+      <c r="E397" s="2" t="inlineStr">
+        <is>
+          <t>ˈaʊɾə</t>
+        </is>
+      </c>
+      <c r="F397" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G397" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="2" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="B398" s="2" t="inlineStr">
+        <is>
+          <t>OF vira â</t>
+        </is>
+      </c>
+      <c r="C398" s="2" t="inlineStr">
+        <is>
+          <t>a lotta (a lot of)</t>
+        </is>
+      </c>
+      <c r="D398" s="2" t="inlineStr">
+        <is>
+          <t>â-LÁ-ɾâ</t>
+        </is>
+      </c>
+      <c r="E398" s="2" t="inlineStr">
+        <is>
+          <t>əˈlɑɾə</t>
+        </is>
+      </c>
+      <c r="F398" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G398" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="2" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="B399" s="2" t="inlineStr">
+        <is>
+          <t>HAVE vira â</t>
+        </is>
+      </c>
+      <c r="C399" s="2" t="inlineStr">
+        <is>
+          <t>shoulda (should have)</t>
+        </is>
+      </c>
+      <c r="D399" s="2" t="inlineStr">
+        <is>
+          <t>SHU-ɾâ</t>
+        </is>
+      </c>
+      <c r="E399" s="2" t="inlineStr">
+        <is>
+          <t>ˈʃʊɾə</t>
+        </is>
+      </c>
+      <c r="F399" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G399" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="2" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="B400" s="2" t="inlineStr">
+        <is>
+          <t>HAVE vira â</t>
+        </is>
+      </c>
+      <c r="C400" s="2" t="inlineStr">
+        <is>
+          <t>coulda (could have)</t>
+        </is>
+      </c>
+      <c r="D400" s="2" t="inlineStr">
+        <is>
+          <t>KU-ɾâ</t>
+        </is>
+      </c>
+      <c r="E400" s="2" t="inlineStr">
+        <is>
+          <t>ˈkʊɾə</t>
+        </is>
+      </c>
+      <c r="F400" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G400" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="2" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="B401" s="2" t="inlineStr">
+        <is>
+          <t>HAVE vira â</t>
+        </is>
+      </c>
+      <c r="C401" s="2" t="inlineStr">
+        <is>
+          <t>woulda (would have)</t>
+        </is>
+      </c>
+      <c r="D401" s="2" t="inlineStr">
+        <is>
+          <t>WU-ɾâ</t>
+        </is>
+      </c>
+      <c r="E401" s="2" t="inlineStr">
+        <is>
+          <t>ˈwʊɾə</t>
+        </is>
+      </c>
+      <c r="F401" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G401" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="2" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="B402" s="2" t="inlineStr">
+        <is>
+          <t>HAVE vira â</t>
+        </is>
+      </c>
+      <c r="C402" s="2" t="inlineStr">
+        <is>
+          <t>musta (must have)</t>
+        </is>
+      </c>
+      <c r="D402" s="2" t="inlineStr">
+        <is>
+          <t>MÂS-tâ</t>
+        </is>
+      </c>
+      <c r="E402" s="2" t="inlineStr">
+        <is>
+          <t>ˈmʌstə</t>
+        </is>
+      </c>
+      <c r="F402" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G402" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="2" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="B403" s="2" t="inlineStr">
+        <is>
+          <t>Outras</t>
+        </is>
+      </c>
+      <c r="C403" s="2" t="inlineStr">
+        <is>
+          <t>lemme (let me)</t>
+        </is>
+      </c>
+      <c r="D403" s="2" t="inlineStr">
+        <is>
+          <t>LÉ-mi</t>
+        </is>
+      </c>
+      <c r="E403" s="2" t="inlineStr">
+        <is>
+          <t>ˈlɛmi</t>
+        </is>
+      </c>
+      <c r="F403" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+      <c r="G403" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="2" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="B404" s="2" t="inlineStr">
+        <is>
+          <t>Outras</t>
+        </is>
+      </c>
+      <c r="C404" s="2" t="inlineStr">
+        <is>
+          <t>gimme (give me)</t>
+        </is>
+      </c>
+      <c r="D404" s="2" t="inlineStr">
+        <is>
+          <t>GI-mi</t>
+        </is>
+      </c>
+      <c r="E404" s="2" t="inlineStr">
+        <is>
+          <t>ˈɡɪmi</t>
+        </is>
+      </c>
+      <c r="F404" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+      <c r="G404" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="2" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="B405" s="2" t="inlineStr">
+        <is>
+          <t>Outras</t>
+        </is>
+      </c>
+      <c r="C405" s="2" t="inlineStr">
+        <is>
+          <t>dunno (don't know)</t>
+        </is>
+      </c>
+      <c r="D405" s="2" t="inlineStr">
+        <is>
+          <t>dâ-NÔU</t>
+        </is>
+      </c>
+      <c r="E405" s="2" t="inlineStr">
+        <is>
+          <t>dəˈnoʊ</t>
+        </is>
+      </c>
+      <c r="F405" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+      <c r="G405" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="2" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="B406" s="2" t="inlineStr">
+        <is>
+          <t>Outras</t>
+        </is>
+      </c>
+      <c r="C406" s="2" t="inlineStr">
+        <is>
+          <t>y'all (you all)</t>
+        </is>
+      </c>
+      <c r="D406" s="2" t="inlineStr">
+        <is>
+          <t>YÁL</t>
+        </is>
+      </c>
+      <c r="E406" s="2" t="inlineStr">
+        <is>
+          <t>jɑl</t>
+        </is>
+      </c>
+      <c r="F406" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+      <c r="G406" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="2" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="B407" s="2" t="inlineStr">
+        <is>
+          <t>Outras</t>
+        </is>
+      </c>
+      <c r="C407" s="2" t="inlineStr">
+        <is>
+          <t>ain't (am not / isn't)</t>
+        </is>
+      </c>
+      <c r="D407" s="2" t="inlineStr">
+        <is>
+          <t>ÊINT</t>
+        </is>
+      </c>
+      <c r="E407" s="2" t="inlineStr">
+        <is>
+          <t>eɪnt</t>
+        </is>
+      </c>
+      <c r="F407" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G407" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="2" t="inlineStr">
+        <is>
+          <t>JUNC</t>
+        </is>
+      </c>
+      <c r="B408" s="2" t="inlineStr">
+        <is>
+          <t>t + you = tchâ</t>
+        </is>
+      </c>
+      <c r="C408" s="2" t="inlineStr">
+        <is>
+          <t>whatcha (what are you)</t>
+        </is>
+      </c>
+      <c r="D408" s="2" t="inlineStr">
+        <is>
+          <t>WÁ-tchâ</t>
+        </is>
+      </c>
+      <c r="E408" s="2" t="inlineStr">
+        <is>
+          <t>ˈwɑtʃə</t>
+        </is>
+      </c>
+      <c r="F408" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+      <c r="G408" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="2" t="inlineStr">
+        <is>
+          <t>JUNC</t>
+        </is>
+      </c>
+      <c r="B409" s="2" t="inlineStr">
+        <is>
+          <t>t + you = tchâ</t>
+        </is>
+      </c>
+      <c r="C409" s="2" t="inlineStr">
+        <is>
+          <t>gotcha (got you)</t>
+        </is>
+      </c>
+      <c r="D409" s="2" t="inlineStr">
+        <is>
+          <t>GÁ-tchâ</t>
+        </is>
+      </c>
+      <c r="E409" s="2" t="inlineStr">
+        <is>
+          <t>ˈɡɑtʃə</t>
+        </is>
+      </c>
+      <c r="F409" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G409" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="2" t="inlineStr">
+        <is>
+          <t>JUNC</t>
+        </is>
+      </c>
+      <c r="B410" s="2" t="inlineStr">
+        <is>
+          <t>t + you = tchâ</t>
+        </is>
+      </c>
+      <c r="C410" s="2" t="inlineStr">
+        <is>
+          <t>don'tcha (don't you)</t>
+        </is>
+      </c>
+      <c r="D410" s="2" t="inlineStr">
+        <is>
+          <t>DÔUN-tchâ</t>
+        </is>
+      </c>
+      <c r="E410" s="2" t="inlineStr">
+        <is>
+          <t>ˈdoʊntʃə</t>
+        </is>
+      </c>
+      <c r="F410" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G410" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="2" t="inlineStr">
+        <is>
+          <t>JUNC</t>
+        </is>
+      </c>
+      <c r="B411" s="2" t="inlineStr">
+        <is>
+          <t>t + you = tchâ</t>
+        </is>
+      </c>
+      <c r="C411" s="2" t="inlineStr">
+        <is>
+          <t>meet you</t>
+        </is>
+      </c>
+      <c r="D411" s="2" t="inlineStr">
+        <is>
+          <t>MII-tchâ</t>
+        </is>
+      </c>
+      <c r="E411" s="2" t="inlineStr">
+        <is>
+          <t>ˈmitʃə</t>
+        </is>
+      </c>
+      <c r="F411" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G411" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="2" t="inlineStr">
+        <is>
+          <t>JUNC</t>
+        </is>
+      </c>
+      <c r="B412" s="2" t="inlineStr">
+        <is>
+          <t>t + you = tchâ</t>
+        </is>
+      </c>
+      <c r="C412" s="2" t="inlineStr">
+        <is>
+          <t>last year</t>
+        </is>
+      </c>
+      <c r="D412" s="2" t="inlineStr">
+        <is>
+          <t>læs-TCHIR</t>
+        </is>
+      </c>
+      <c r="E412" s="2" t="inlineStr">
+        <is>
+          <t>ˌlæsˈtʃɪr</t>
+        </is>
+      </c>
+      <c r="F412" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G412" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="2" t="inlineStr">
+        <is>
+          <t>JUNC</t>
+        </is>
+      </c>
+      <c r="B413" s="2" t="inlineStr">
+        <is>
+          <t>d + you = djâ</t>
+        </is>
+      </c>
+      <c r="C413" s="2" t="inlineStr">
+        <is>
+          <t>didja (did you)</t>
+        </is>
+      </c>
+      <c r="D413" s="2" t="inlineStr">
+        <is>
+          <t>DI-djâ</t>
+        </is>
+      </c>
+      <c r="E413" s="2" t="inlineStr">
+        <is>
+          <t>ˈdɪdʒə</t>
+        </is>
+      </c>
+      <c r="F413" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G413" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="2" t="inlineStr">
+        <is>
+          <t>JUNC</t>
+        </is>
+      </c>
+      <c r="B414" s="2" t="inlineStr">
+        <is>
+          <t>d + you = djâ</t>
+        </is>
+      </c>
+      <c r="C414" s="2" t="inlineStr">
+        <is>
+          <t>wouldja (would you)</t>
+        </is>
+      </c>
+      <c r="D414" s="2" t="inlineStr">
+        <is>
+          <t>WU-djâ</t>
+        </is>
+      </c>
+      <c r="E414" s="2" t="inlineStr">
+        <is>
+          <t>ˈwʊdʒə</t>
+        </is>
+      </c>
+      <c r="F414" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G414" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="2" t="inlineStr">
+        <is>
+          <t>JUNC</t>
+        </is>
+      </c>
+      <c r="B415" s="2" t="inlineStr">
+        <is>
+          <t>d + you = djâ</t>
+        </is>
+      </c>
+      <c r="C415" s="2" t="inlineStr">
+        <is>
+          <t>couldja (could you)</t>
+        </is>
+      </c>
+      <c r="D415" s="2" t="inlineStr">
+        <is>
+          <t>KU-djâ</t>
+        </is>
+      </c>
+      <c r="E415" s="2" t="inlineStr">
+        <is>
+          <t>ˈkʊdʒə</t>
+        </is>
+      </c>
+      <c r="F415" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G415" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="2" t="inlineStr">
+        <is>
+          <t>JUNC</t>
+        </is>
+      </c>
+      <c r="B416" s="2" t="inlineStr">
+        <is>
+          <t>d + you = djâ</t>
+        </is>
+      </c>
+      <c r="C416" s="2" t="inlineStr">
+        <is>
+          <t>need you</t>
+        </is>
+      </c>
+      <c r="D416" s="2" t="inlineStr">
+        <is>
+          <t>NII-djâ</t>
+        </is>
+      </c>
+      <c r="E416" s="2" t="inlineStr">
+        <is>
+          <t>ˈnidʒə</t>
+        </is>
+      </c>
+      <c r="F416" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G416" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="2" t="inlineStr">
+        <is>
+          <t>FRACAS</t>
+        </is>
+      </c>
+      <c r="B417" s="2" t="n"/>
+      <c r="C417" s="2" t="inlineStr">
+        <is>
+          <t>to</t>
+        </is>
+      </c>
+      <c r="D417" s="2" t="inlineStr">
+        <is>
+          <t>tâ (forte: TUU)</t>
+        </is>
+      </c>
+      <c r="E417" s="2" t="inlineStr">
+        <is>
+          <t>tə</t>
+        </is>
+      </c>
+      <c r="F417" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G417" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="2" t="inlineStr">
+        <is>
+          <t>FRACAS</t>
+        </is>
+      </c>
+      <c r="B418" s="2" t="n"/>
+      <c r="C418" s="2" t="inlineStr">
+        <is>
+          <t>for</t>
+        </is>
+      </c>
+      <c r="D418" s="2" t="inlineStr">
+        <is>
+          <t>fâr (forte: FÓR)</t>
+        </is>
+      </c>
+      <c r="E418" s="2" t="inlineStr">
+        <is>
+          <t>fɚ</t>
+        </is>
+      </c>
+      <c r="F418" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G418" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="2" t="inlineStr">
+        <is>
+          <t>FRACAS</t>
+        </is>
+      </c>
+      <c r="B419" s="2" t="n"/>
+      <c r="C419" s="2" t="inlineStr">
+        <is>
+          <t>and</t>
+        </is>
+      </c>
+      <c r="D419" s="2" t="inlineStr">
+        <is>
+          <t>ân (forte: ÆND)</t>
+        </is>
+      </c>
+      <c r="E419" s="2" t="inlineStr">
+        <is>
+          <t>ən</t>
+        </is>
+      </c>
+      <c r="F419" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G419" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="2" t="inlineStr">
+        <is>
+          <t>FRACAS</t>
+        </is>
+      </c>
+      <c r="B420" s="2" t="n"/>
+      <c r="C420" s="2" t="inlineStr">
+        <is>
+          <t>of</t>
+        </is>
+      </c>
+      <c r="D420" s="2" t="inlineStr">
+        <is>
+          <t>âv (forte: ÂV)</t>
+        </is>
+      </c>
+      <c r="E420" s="2" t="inlineStr">
+        <is>
+          <t>əv</t>
+        </is>
+      </c>
+      <c r="F420" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G420" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" s="2" t="inlineStr">
+        <is>
+          <t>FRACAS</t>
+        </is>
+      </c>
+      <c r="B421" s="2" t="n"/>
+      <c r="C421" s="2" t="inlineStr">
+        <is>
+          <t>you</t>
+        </is>
+      </c>
+      <c r="D421" s="2" t="inlineStr">
+        <is>
+          <t>yâ (forte: YUU)</t>
+        </is>
+      </c>
+      <c r="E421" s="2" t="inlineStr">
+        <is>
+          <t>jə</t>
+        </is>
+      </c>
+      <c r="F421" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G421" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="2" t="inlineStr">
+        <is>
+          <t>FRACAS</t>
+        </is>
+      </c>
+      <c r="B422" s="2" t="n"/>
+      <c r="C422" s="2" t="inlineStr">
+        <is>
+          <t>your</t>
+        </is>
+      </c>
+      <c r="D422" s="2" t="inlineStr">
+        <is>
+          <t>yâr (forte: YUR)</t>
+        </is>
+      </c>
+      <c r="E422" s="2" t="inlineStr">
+        <is>
+          <t>jɚ</t>
+        </is>
+      </c>
+      <c r="F422" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G422" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="2" t="inlineStr">
+        <is>
+          <t>FRACAS</t>
+        </is>
+      </c>
+      <c r="B423" s="2" t="n"/>
+      <c r="C423" s="2" t="inlineStr">
+        <is>
+          <t>them</t>
+        </is>
+      </c>
+      <c r="D423" s="2" t="inlineStr">
+        <is>
+          <t>âm (forte: DHÉM)</t>
+        </is>
+      </c>
+      <c r="E423" s="2" t="inlineStr">
+        <is>
+          <t>əm</t>
+        </is>
+      </c>
+      <c r="F423" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G423" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="2" t="inlineStr">
+        <is>
+          <t>FRACAS</t>
+        </is>
+      </c>
+      <c r="B424" s="2" t="n"/>
+      <c r="C424" s="2" t="inlineStr">
+        <is>
+          <t>him</t>
+        </is>
+      </c>
+      <c r="D424" s="2" t="inlineStr">
+        <is>
+          <t>im (forte: HIM)</t>
+        </is>
+      </c>
+      <c r="E424" s="2" t="inlineStr">
+        <is>
+          <t>ɪm</t>
+        </is>
+      </c>
+      <c r="F424" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G424" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="2" t="inlineStr">
+        <is>
+          <t>FRACAS</t>
+        </is>
+      </c>
+      <c r="B425" s="2" t="n"/>
+      <c r="C425" s="2" t="inlineStr">
+        <is>
+          <t>her</t>
+        </is>
+      </c>
+      <c r="D425" s="2" t="inlineStr">
+        <is>
+          <t>âr (forte: HÂR)</t>
+        </is>
+      </c>
+      <c r="E425" s="2" t="inlineStr">
+        <is>
+          <t>ɚ</t>
+        </is>
+      </c>
+      <c r="F425" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G425" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="2" t="inlineStr">
+        <is>
+          <t>FRACAS</t>
+        </is>
+      </c>
+      <c r="B426" s="2" t="n"/>
+      <c r="C426" s="2" t="inlineStr">
+        <is>
+          <t>have</t>
+        </is>
+      </c>
+      <c r="D426" s="2" t="inlineStr">
+        <is>
+          <t>âv (forte: HÆV)</t>
+        </is>
+      </c>
+      <c r="E426" s="2" t="inlineStr">
+        <is>
+          <t>əv</t>
+        </is>
+      </c>
+      <c r="F426" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G426" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="2" t="inlineStr">
+        <is>
+          <t>FRACAS</t>
+        </is>
+      </c>
+      <c r="B427" s="2" t="n"/>
+      <c r="C427" s="2" t="inlineStr">
+        <is>
+          <t>can</t>
+        </is>
+      </c>
+      <c r="D427" s="2" t="inlineStr">
+        <is>
+          <t>kân (forte: KÆN)</t>
+        </is>
+      </c>
+      <c r="E427" s="2" t="inlineStr">
+        <is>
+          <t>kən</t>
+        </is>
+      </c>
+      <c r="F427" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G427" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="2" t="inlineStr">
+        <is>
+          <t>FRACAS</t>
+        </is>
+      </c>
+      <c r="B428" s="2" t="n"/>
+      <c r="C428" s="2" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D428" s="2" t="inlineStr">
+        <is>
+          <t>ât (forte: ÆT)</t>
+        </is>
+      </c>
+      <c r="E428" s="2" t="inlineStr">
+        <is>
+          <t>ət</t>
+        </is>
+      </c>
+      <c r="F428" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G428" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="2" t="inlineStr">
+        <is>
+          <t>FRACAS</t>
+        </is>
+      </c>
+      <c r="B429" s="2" t="n"/>
+      <c r="C429" s="2" t="inlineStr">
+        <is>
+          <t>was</t>
+        </is>
+      </c>
+      <c r="D429" s="2" t="inlineStr">
+        <is>
+          <t>wâz (forte: WÂZ)</t>
+        </is>
+      </c>
+      <c r="E429" s="2" t="inlineStr">
+        <is>
+          <t>wəz</t>
+        </is>
+      </c>
+      <c r="F429" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G429" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="2" t="inlineStr">
+        <is>
+          <t>CONECT</t>
+        </is>
+      </c>
+      <c r="B430" s="2" t="inlineStr">
+        <is>
+          <t>Causa e consequência: porque · então · portanto</t>
+        </is>
+      </c>
+      <c r="C430" s="2" t="inlineStr">
+        <is>
+          <t>because</t>
+        </is>
+      </c>
+      <c r="D430" s="2" t="inlineStr">
+        <is>
+          <t>bi-KÁZ (rápido: KÂZ)</t>
+        </is>
+      </c>
+      <c r="E430" s="2" t="inlineStr">
+        <is>
+          <t>bɪˈkɑz</t>
+        </is>
+      </c>
+      <c r="F430" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+      <c r="G430" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="2" t="inlineStr">
+        <is>
+          <t>CONECT</t>
+        </is>
+      </c>
+      <c r="B431" s="2" t="inlineStr">
+        <is>
+          <t>Causa e consequência: porque · então · portanto</t>
+        </is>
+      </c>
+      <c r="C431" s="2" t="inlineStr">
+        <is>
+          <t>so</t>
+        </is>
+      </c>
+      <c r="D431" s="2" t="inlineStr">
+        <is>
+          <t>SÔU</t>
+        </is>
+      </c>
+      <c r="E431" s="2" t="inlineStr">
+        <is>
+          <t>soʊ</t>
+        </is>
+      </c>
+      <c r="F431" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+      <c r="G431" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="2" t="inlineStr">
+        <is>
+          <t>CONECT</t>
+        </is>
+      </c>
+      <c r="B432" s="2" t="inlineStr">
+        <is>
+          <t>Causa e consequência: porque · então · portanto</t>
+        </is>
+      </c>
+      <c r="C432" s="2" t="inlineStr">
+        <is>
+          <t>therefore</t>
+        </is>
+      </c>
+      <c r="D432" s="2" t="inlineStr">
+        <is>
+          <t>DHÉR-fór</t>
+        </is>
+      </c>
+      <c r="E432" s="2" t="inlineStr">
+        <is>
+          <t>ˈðɛrfɔr</t>
+        </is>
+      </c>
+      <c r="F432" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G432" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="2" t="inlineStr">
+        <is>
+          <t>CONECT</t>
+        </is>
+      </c>
+      <c r="B433" s="2" t="inlineStr">
+        <is>
+          <t>Contraste: mas · embora · porém · enquanto</t>
+        </is>
+      </c>
+      <c r="C433" s="2" t="inlineStr">
+        <is>
+          <t>but</t>
+        </is>
+      </c>
+      <c r="D433" s="2" t="inlineStr">
+        <is>
+          <t>BÂT</t>
+        </is>
+      </c>
+      <c r="E433" s="2" t="inlineStr">
+        <is>
+          <t>bʌt</t>
+        </is>
+      </c>
+      <c r="F433" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+      <c r="G433" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" s="2" t="inlineStr">
+        <is>
+          <t>CONECT</t>
+        </is>
+      </c>
+      <c r="B434" s="2" t="inlineStr">
+        <is>
+          <t>Contraste: mas · embora · porém · enquanto</t>
+        </is>
+      </c>
+      <c r="C434" s="2" t="inlineStr">
+        <is>
+          <t>although</t>
+        </is>
+      </c>
+      <c r="D434" s="2" t="inlineStr">
+        <is>
+          <t>ál-DHÔU</t>
+        </is>
+      </c>
+      <c r="E434" s="2" t="inlineStr">
+        <is>
+          <t>ɑlˈðoʊ</t>
+        </is>
+      </c>
+      <c r="F434" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+      <c r="G434" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="2" t="inlineStr">
+        <is>
+          <t>CONECT</t>
+        </is>
+      </c>
+      <c r="B435" s="2" t="inlineStr">
+        <is>
+          <t>Contraste: mas · embora · porém · enquanto</t>
+        </is>
+      </c>
+      <c r="C435" s="2" t="inlineStr">
+        <is>
+          <t>though</t>
+        </is>
+      </c>
+      <c r="D435" s="2" t="inlineStr">
+        <is>
+          <t>DHÔU</t>
+        </is>
+      </c>
+      <c r="E435" s="2" t="inlineStr">
+        <is>
+          <t>ðoʊ</t>
+        </is>
+      </c>
+      <c r="F435" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G435" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="2" t="inlineStr">
+        <is>
+          <t>CONECT</t>
+        </is>
+      </c>
+      <c r="B436" s="2" t="inlineStr">
+        <is>
+          <t>Contraste: mas · embora · porém · enquanto</t>
+        </is>
+      </c>
+      <c r="C436" s="2" t="inlineStr">
+        <is>
+          <t>however</t>
+        </is>
+      </c>
+      <c r="D436" s="2" t="inlineStr">
+        <is>
+          <t>háu-É-vâr</t>
+        </is>
+      </c>
+      <c r="E436" s="2" t="inlineStr">
+        <is>
+          <t>haʊˈɛvɚ</t>
+        </is>
+      </c>
+      <c r="F436" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+      <c r="G436" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="2" t="inlineStr">
+        <is>
+          <t>CONECT</t>
+        </is>
+      </c>
+      <c r="B437" s="2" t="inlineStr">
+        <is>
+          <t>Contraste: mas · embora · porém · enquanto</t>
+        </is>
+      </c>
+      <c r="C437" s="2" t="inlineStr">
+        <is>
+          <t>whereas</t>
+        </is>
+      </c>
+      <c r="D437" s="2" t="inlineStr">
+        <is>
+          <t>wér-ÆZ</t>
+        </is>
+      </c>
+      <c r="E437" s="2" t="inlineStr">
+        <is>
+          <t>wɛrˈæz</t>
+        </is>
+      </c>
+      <c r="F437" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G437" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="2" t="inlineStr">
+        <is>
+          <t>CONECT</t>
+        </is>
+      </c>
+      <c r="B438" s="2" t="inlineStr">
+        <is>
+          <t>Adicionar: também · além disso · de fato</t>
+        </is>
+      </c>
+      <c r="C438" s="2" t="inlineStr">
+        <is>
+          <t>also</t>
+        </is>
+      </c>
+      <c r="D438" s="2" t="inlineStr">
+        <is>
+          <t>ÁL-sôu</t>
+        </is>
+      </c>
+      <c r="E438" s="2" t="inlineStr">
+        <is>
+          <t>ˈɑlsoʊ</t>
+        </is>
+      </c>
+      <c r="F438" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+      <c r="G438" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" s="2" t="inlineStr">
+        <is>
+          <t>CONECT</t>
+        </is>
+      </c>
+      <c r="B439" s="2" t="inlineStr">
+        <is>
+          <t>Adicionar: também · além disso · de fato</t>
+        </is>
+      </c>
+      <c r="C439" s="2" t="inlineStr">
+        <is>
+          <t>besides</t>
+        </is>
+      </c>
+      <c r="D439" s="2" t="inlineStr">
+        <is>
+          <t>bi-SÁIDZ</t>
+        </is>
+      </c>
+      <c r="E439" s="2" t="inlineStr">
+        <is>
+          <t>bɪˈsaɪdz</t>
+        </is>
+      </c>
+      <c r="F439" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G439" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="2" t="inlineStr">
+        <is>
+          <t>CONECT</t>
+        </is>
+      </c>
+      <c r="B440" s="2" t="inlineStr">
+        <is>
+          <t>Adicionar: também · além disso · de fato</t>
+        </is>
+      </c>
+      <c r="C440" s="2" t="inlineStr">
+        <is>
+          <t>in fact</t>
+        </is>
+      </c>
+      <c r="D440" s="2" t="inlineStr">
+        <is>
+          <t>in-FÆKT</t>
+        </is>
+      </c>
+      <c r="E440" s="2" t="inlineStr">
+        <is>
+          <t>ɪnˈfækt</t>
+        </is>
+      </c>
+      <c r="F440" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G440" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="2" t="inlineStr">
+        <is>
+          <t>CONECT</t>
+        </is>
+      </c>
+      <c r="B441" s="2" t="inlineStr">
+        <is>
+          <t>Assunto: na verdade · enfim · aliás</t>
+        </is>
+      </c>
+      <c r="C441" s="2" t="inlineStr">
+        <is>
+          <t>actually</t>
+        </is>
+      </c>
+      <c r="D441" s="2" t="inlineStr">
+        <is>
+          <t>ÆK-tchuu-â-li (rápido: ÆK-shâ-li)</t>
+        </is>
+      </c>
+      <c r="E441" s="2" t="inlineStr">
+        <is>
+          <t>ˈæktʃuəli</t>
+        </is>
+      </c>
+      <c r="F441" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+      <c r="G441" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="2" t="inlineStr">
+        <is>
+          <t>CONECT</t>
+        </is>
+      </c>
+      <c r="B442" s="2" t="inlineStr">
+        <is>
+          <t>Assunto: na verdade · enfim · aliás</t>
+        </is>
+      </c>
+      <c r="C442" s="2" t="inlineStr">
+        <is>
+          <t>anyway</t>
+        </is>
+      </c>
+      <c r="D442" s="2" t="inlineStr">
+        <is>
+          <t>É-ni-wêi</t>
+        </is>
+      </c>
+      <c r="E442" s="2" t="inlineStr">
+        <is>
+          <t>ˈɛniweɪ</t>
+        </is>
+      </c>
+      <c r="F442" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+      <c r="G442" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="2" t="inlineStr">
+        <is>
+          <t>CONECT</t>
+        </is>
+      </c>
+      <c r="B443" s="2" t="inlineStr">
+        <is>
+          <t>Assunto: na verdade · enfim · aliás</t>
+        </is>
+      </c>
+      <c r="C443" s="2" t="inlineStr">
+        <is>
+          <t>by the way</t>
+        </is>
+      </c>
+      <c r="D443" s="2" t="inlineStr">
+        <is>
+          <t>bái-dhâ-WÊI</t>
+        </is>
+      </c>
+      <c r="E443" s="2" t="inlineStr">
+        <is>
+          <t>ˌbaɪ ðə ˈweɪ</t>
+        </is>
+      </c>
+      <c r="F443" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+      <c r="G443" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="2" t="inlineStr">
+        <is>
+          <t>CONECT</t>
+        </is>
+      </c>
+      <c r="B444" s="2" t="inlineStr">
+        <is>
+          <t>Alternativa: em vez disso · senão · a menos que</t>
+        </is>
+      </c>
+      <c r="C444" s="2" t="inlineStr">
+        <is>
+          <t>instead</t>
+        </is>
+      </c>
+      <c r="D444" s="2" t="inlineStr">
+        <is>
+          <t>in-STÉD</t>
+        </is>
+      </c>
+      <c r="E444" s="2" t="inlineStr">
+        <is>
+          <t>ɪnˈstɛd</t>
+        </is>
+      </c>
+      <c r="F444" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+      <c r="G444" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="2" t="inlineStr">
+        <is>
+          <t>CONECT</t>
+        </is>
+      </c>
+      <c r="B445" s="2" t="inlineStr">
+        <is>
+          <t>Alternativa: em vez disso · senão · a menos que</t>
+        </is>
+      </c>
+      <c r="C445" s="2" t="inlineStr">
+        <is>
+          <t>otherwise</t>
+        </is>
+      </c>
+      <c r="D445" s="2" t="inlineStr">
+        <is>
+          <t>Â-dhâr-wáiz</t>
+        </is>
+      </c>
+      <c r="E445" s="2" t="inlineStr">
+        <is>
+          <t>ˈʌðɚwaɪz</t>
+        </is>
+      </c>
+      <c r="F445" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G445" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="2" t="inlineStr">
+        <is>
+          <t>CONECT</t>
+        </is>
+      </c>
+      <c r="B446" s="2" t="inlineStr">
+        <is>
+          <t>Alternativa: em vez disso · senão · a menos que</t>
+        </is>
+      </c>
+      <c r="C446" s="2" t="inlineStr">
+        <is>
+          <t>unless</t>
+        </is>
+      </c>
+      <c r="D446" s="2" t="inlineStr">
+        <is>
+          <t>ân-LÉS</t>
+        </is>
+      </c>
+      <c r="E446" s="2" t="inlineStr">
+        <is>
+          <t>ənˈlɛs</t>
+        </is>
+      </c>
+      <c r="F446" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G446" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="2" t="inlineStr">
+        <is>
+          <t>EFINAL</t>
+        </is>
+      </c>
+      <c r="B447" s="2" t="n"/>
+      <c r="C447" s="2" t="inlineStr">
+        <is>
+          <t>recipe</t>
+        </is>
+      </c>
+      <c r="D447" s="2" t="inlineStr">
+        <is>
+          <t>RÉ-sâ-pi</t>
+        </is>
+      </c>
+      <c r="E447" s="2" t="inlineStr">
+        <is>
+          <t>ˈrɛsəpi</t>
+        </is>
+      </c>
+      <c r="F447" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+      <c r="G447" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="2" t="inlineStr">
+        <is>
+          <t>EFINAL</t>
+        </is>
+      </c>
+      <c r="B448" s="2" t="n"/>
+      <c r="C448" s="2" t="inlineStr">
+        <is>
+          <t>acne</t>
+        </is>
+      </c>
+      <c r="D448" s="2" t="inlineStr">
+        <is>
+          <t>ÆK-ni</t>
+        </is>
+      </c>
+      <c r="E448" s="2" t="inlineStr">
+        <is>
+          <t>ˈækni</t>
+        </is>
+      </c>
+      <c r="F448" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G448" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" s="2" t="inlineStr">
+        <is>
+          <t>EFINAL</t>
+        </is>
+      </c>
+      <c r="B449" s="2" t="n"/>
+      <c r="C449" s="2" t="inlineStr">
+        <is>
+          <t>karate</t>
+        </is>
+      </c>
+      <c r="D449" s="2" t="inlineStr">
+        <is>
+          <t>kâ-RÁ-ɾi</t>
+        </is>
+      </c>
+      <c r="E449" s="2" t="inlineStr">
+        <is>
+          <t>kəˈrɑɾi</t>
+        </is>
+      </c>
+      <c r="F449" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G449" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="2" t="inlineStr">
+        <is>
+          <t>EFINAL</t>
+        </is>
+      </c>
+      <c r="B450" s="2" t="n"/>
+      <c r="C450" s="2" t="inlineStr">
+        <is>
+          <t>sesame</t>
+        </is>
+      </c>
+      <c r="D450" s="2" t="inlineStr">
+        <is>
+          <t>SÉ-sâ-mi</t>
+        </is>
+      </c>
+      <c r="E450" s="2" t="inlineStr">
+        <is>
+          <t>ˈsɛsəmi</t>
+        </is>
+      </c>
+      <c r="F450" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G450" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="2" t="inlineStr">
+        <is>
+          <t>EFINAL</t>
+        </is>
+      </c>
+      <c r="B451" s="2" t="n"/>
+      <c r="C451" s="2" t="inlineStr">
+        <is>
+          <t>apostrophe</t>
+        </is>
+      </c>
+      <c r="D451" s="2" t="inlineStr">
+        <is>
+          <t>â-PÁS-trâ-fi</t>
+        </is>
+      </c>
+      <c r="E451" s="2" t="inlineStr">
+        <is>
+          <t>əˈpɑstrəfi</t>
+        </is>
+      </c>
+      <c r="F451" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G451" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="2" t="inlineStr">
+        <is>
+          <t>EFINAL</t>
+        </is>
+      </c>
+      <c r="B452" s="2" t="n"/>
+      <c r="C452" s="2" t="inlineStr">
+        <is>
+          <t>catastrophe</t>
+        </is>
+      </c>
+      <c r="D452" s="2" t="inlineStr">
+        <is>
+          <t>kâ-TÆS-trâ-fi</t>
+        </is>
+      </c>
+      <c r="E452" s="2" t="inlineStr">
+        <is>
+          <t>kəˈtæstrəfi</t>
+        </is>
+      </c>
+      <c r="F452" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G452" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" s="2" t="inlineStr">
+        <is>
+          <t>EFINAL</t>
+        </is>
+      </c>
+      <c r="B453" s="2" t="n"/>
+      <c r="C453" s="2" t="inlineStr">
+        <is>
+          <t>coyote</t>
+        </is>
+      </c>
+      <c r="D453" s="2" t="inlineStr">
+        <is>
+          <t>kái-ÔU-ɾi</t>
+        </is>
+      </c>
+      <c r="E453" s="2" t="inlineStr">
+        <is>
+          <t>kaɪˈoʊɾi</t>
+        </is>
+      </c>
+      <c r="F453" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G453" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="2" t="inlineStr">
+        <is>
+          <t>EFINAL</t>
+        </is>
+      </c>
+      <c r="B454" s="2" t="n"/>
+      <c r="C454" s="2" t="inlineStr">
+        <is>
+          <t>adobe</t>
+        </is>
+      </c>
+      <c r="D454" s="2" t="inlineStr">
+        <is>
+          <t>â-DÔU-bi</t>
+        </is>
+      </c>
+      <c r="E454" s="2" t="inlineStr">
+        <is>
+          <t>əˈdoʊbi</t>
+        </is>
+      </c>
+      <c r="F454" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G454" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="2" t="inlineStr">
+        <is>
+          <t>GRAF</t>
+        </is>
+      </c>
+      <c r="B455" s="2" t="n"/>
+      <c r="C455" s="2" t="inlineStr">
+        <is>
+          <t>clothes</t>
+        </is>
+      </c>
+      <c r="D455" s="2" t="inlineStr">
+        <is>
+          <t>KLÔUDHZ (rápido: KLÔUZ)</t>
+        </is>
+      </c>
+      <c r="E455" s="2" t="inlineStr">
+        <is>
+          <t>kloʊðz</t>
+        </is>
+      </c>
+      <c r="F455" s="2" t="inlineStr">
+        <is>
+          <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+      <c r="G455" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="2" t="inlineStr">
+        <is>
+          <t>GRAF</t>
+        </is>
+      </c>
+      <c r="B456" s="2" t="n"/>
+      <c r="C456" s="2" t="inlineStr">
+        <is>
+          <t>colonel</t>
+        </is>
+      </c>
+      <c r="D456" s="2" t="inlineStr">
+        <is>
+          <t>KÂR-nâl</t>
+        </is>
+      </c>
+      <c r="E456" s="2" t="inlineStr">
+        <is>
+          <t>ˈkɝnəl</t>
+        </is>
+      </c>
+      <c r="F456" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G456" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" s="2" t="inlineStr">
+        <is>
+          <t>GRAF</t>
+        </is>
+      </c>
+      <c r="B457" s="2" t="n"/>
+      <c r="C457" s="2" t="inlineStr">
+        <is>
+          <t>women</t>
+        </is>
+      </c>
+      <c r="D457" s="2" t="inlineStr">
+        <is>
+          <t>WI-min</t>
+        </is>
+      </c>
+      <c r="E457" s="2" t="inlineStr">
+        <is>
+          <t>ˈwɪmɪn</t>
+        </is>
+      </c>
+      <c r="F457" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G457" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="2" t="inlineStr">
+        <is>
+          <t>GRAF</t>
+        </is>
+      </c>
+      <c r="B458" s="2" t="n"/>
+      <c r="C458" s="2" t="inlineStr">
+        <is>
+          <t>busy</t>
+        </is>
+      </c>
+      <c r="D458" s="2" t="inlineStr">
+        <is>
+          <t>BI-zi</t>
+        </is>
+      </c>
+      <c r="E458" s="2" t="inlineStr">
+        <is>
+          <t>ˈbɪzi</t>
+        </is>
+      </c>
+      <c r="F458" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G458" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" s="2" t="inlineStr">
+        <is>
+          <t>GRAF</t>
+        </is>
+      </c>
+      <c r="B459" s="2" t="n"/>
+      <c r="C459" s="2" t="inlineStr">
+        <is>
+          <t>bury</t>
+        </is>
+      </c>
+      <c r="D459" s="2" t="inlineStr">
+        <is>
+          <t>BÉ-ri</t>
+        </is>
+      </c>
+      <c r="E459" s="2" t="inlineStr">
+        <is>
+          <t>ˈbɛri</t>
+        </is>
+      </c>
+      <c r="F459" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G459" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="2" t="inlineStr">
+        <is>
+          <t>GRAF</t>
+        </is>
+      </c>
+      <c r="B460" s="2" t="n"/>
+      <c r="C460" s="2" t="inlineStr">
+        <is>
+          <t>lettuce</t>
+        </is>
+      </c>
+      <c r="D460" s="2" t="inlineStr">
+        <is>
+          <t>LÉ-ɾis</t>
+        </is>
+      </c>
+      <c r="E460" s="2" t="inlineStr">
+        <is>
+          <t>ˈlɛɾɪs</t>
+        </is>
+      </c>
+      <c r="F460" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G460" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" s="2" t="inlineStr">
+        <is>
+          <t>GRAF</t>
+        </is>
+      </c>
+      <c r="B461" s="2" t="n"/>
+      <c r="C461" s="2" t="inlineStr">
+        <is>
+          <t>choir</t>
+        </is>
+      </c>
+      <c r="D461" s="2" t="inlineStr">
+        <is>
+          <t>KWÁI-âr</t>
+        </is>
+      </c>
+      <c r="E461" s="2" t="inlineStr">
+        <is>
+          <t>ˈkwaɪɚ</t>
+        </is>
+      </c>
+      <c r="F461" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G461" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="2" t="inlineStr">
+        <is>
+          <t>GRAF</t>
+        </is>
+      </c>
+      <c r="B462" s="2" t="n"/>
+      <c r="C462" s="2" t="inlineStr">
+        <is>
+          <t>iron</t>
+        </is>
+      </c>
+      <c r="D462" s="2" t="inlineStr">
+        <is>
+          <t>ÁI-ârn</t>
+        </is>
+      </c>
+      <c r="E462" s="2" t="inlineStr">
+        <is>
+          <t>ˈaɪɚn</t>
+        </is>
+      </c>
+      <c r="F462" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G462" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="2" t="inlineStr">
+        <is>
+          <t>GRAF</t>
+        </is>
+      </c>
+      <c r="B463" s="2" t="n"/>
+      <c r="C463" s="2" t="inlineStr">
+        <is>
+          <t>jewelry</t>
+        </is>
+      </c>
+      <c r="D463" s="2" t="inlineStr">
+        <is>
+          <t>DJUU-âl-ri</t>
+        </is>
+      </c>
+      <c r="E463" s="2" t="inlineStr">
+        <is>
+          <t>ˈdʒuəlri</t>
+        </is>
+      </c>
+      <c r="F463" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G463" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="2" t="inlineStr">
+        <is>
+          <t>GRAF</t>
+        </is>
+      </c>
+      <c r="B464" s="2" t="n"/>
+      <c r="C464" s="2" t="inlineStr">
+        <is>
+          <t>February</t>
+        </is>
+      </c>
+      <c r="D464" s="2" t="inlineStr">
+        <is>
+          <t>FÉB-yuu-é-ri</t>
+        </is>
+      </c>
+      <c r="E464" s="2" t="inlineStr">
+        <is>
+          <t>ˈfɛbjuɛri</t>
+        </is>
+      </c>
+      <c r="F464" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G464" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" s="2" t="inlineStr">
+        <is>
+          <t>GRAF</t>
+        </is>
+      </c>
+      <c r="B465" s="2" t="n"/>
+      <c r="C465" s="2" t="inlineStr">
+        <is>
+          <t>bowl</t>
+        </is>
+      </c>
+      <c r="D465" s="2" t="inlineStr">
+        <is>
+          <t>BÔUL</t>
+        </is>
+      </c>
+      <c r="E465" s="2" t="inlineStr">
+        <is>
+          <t>boʊl</t>
+        </is>
+      </c>
+      <c r="F465" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G465" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="2" t="inlineStr">
+        <is>
+          <t>GRAF</t>
+        </is>
+      </c>
+      <c r="B466" s="2" t="n"/>
+      <c r="C466" s="2" t="inlineStr">
+        <is>
+          <t>says</t>
+        </is>
+      </c>
+      <c r="D466" s="2" t="inlineStr">
+        <is>
+          <t>SÉZ</t>
+        </is>
+      </c>
+      <c r="E466" s="2" t="inlineStr">
+        <is>
+          <t>sɛz</t>
+        </is>
+      </c>
+      <c r="F466" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G466" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="2" t="inlineStr">
+        <is>
+          <t>GRAF</t>
+        </is>
+      </c>
+      <c r="B467" s="2" t="n"/>
+      <c r="C467" s="2" t="inlineStr">
+        <is>
+          <t>minute</t>
+        </is>
+      </c>
+      <c r="D467" s="2" t="inlineStr">
+        <is>
+          <t>MI-nit</t>
+        </is>
+      </c>
+      <c r="E467" s="2" t="inlineStr">
+        <is>
+          <t>ˈmɪnɪt</t>
+        </is>
+      </c>
+      <c r="F467" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G467" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="2" t="inlineStr">
+        <is>
+          <t>GRAF</t>
+        </is>
+      </c>
+      <c r="B468" s="2" t="n"/>
+      <c r="C468" s="2" t="inlineStr">
+        <is>
+          <t>pretty</t>
+        </is>
+      </c>
+      <c r="D468" s="2" t="inlineStr">
+        <is>
+          <t>PRI-ɾi</t>
+        </is>
+      </c>
+      <c r="E468" s="2" t="inlineStr">
+        <is>
+          <t>ˈprɪɾi</t>
+        </is>
+      </c>
+      <c r="F468" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G468" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="2" t="inlineStr">
+        <is>
+          <t>TMUDO</t>
+        </is>
+      </c>
+      <c r="B469" s="2" t="n"/>
+      <c r="C469" s="2" t="inlineStr">
+        <is>
+          <t>mortgage</t>
+        </is>
+      </c>
+      <c r="D469" s="2" t="inlineStr">
+        <is>
+          <t>MÓR-gidj</t>
+        </is>
+      </c>
+      <c r="E469" s="2" t="inlineStr">
+        <is>
+          <t>ˈmɔrɡɪdʒ</t>
+        </is>
+      </c>
+      <c r="F469" s="2" t="inlineStr">
+        <is>
+          <t>Ampliação do post (out/2026)</t>
+        </is>
+      </c>
+      <c r="G469" s="2" t="inlineStr">
         <is>
           <t>treinar</t>
         </is>
@@ -17756,7 +20980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -18786,6 +22010,93 @@
       <c r="F34" s="2" t="inlineStr"/>
       <c r="G34" s="2" t="inlineStr"/>
     </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>can × can't</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>can</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>kân</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>can't</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>KÆNT</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>can × can't</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>I can go</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>ái-kân-GÔU</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>I can't go</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>ái-KÆNT-gôu</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="n"/>
+      <c r="G36" s="2" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>recipe × receipt</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>recipe</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>RÉ-sâ-pi</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>receipt</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>ri-SIIT</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="n"/>
+      <c r="G37" s="2" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -18798,7 +22109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -18910,6 +22221,30 @@
       <c r="B9" s="2" t="inlineStr">
         <is>
           <t>R americano × H (que é o R de "rato" do português).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>can × can't</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Na afirmativa, can é fraco (kân) e o verbo leva a força: I can GO. Na negativa, can't é forte e tem æ, mesmo quando o T some: I CAN'T go.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>recipe × receipt</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>recipe tem o E final que soa (receita); receipt tem o P mudo (recibo).</t>
         </is>
       </c>
     </row>
@@ -20644,12 +23979,12 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>MÆ-gâ-ziin</t>
+          <t>mæ-gâ-ZIIN</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>ˈmæɡəzin</t>
+          <t>ˌmæɡəˈzin</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Inclui reel @marco.essential: grupos -ISM e -CIAN e 7 palavras
Novos grupos ISM (tourism, mechanism, criticism) e CIAN (technician,
electrician); bottle e settle no grupo LE. IPA conferido no Cambridge US.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0138TT66RZLisn7gEtAhCKXA
</commit_message>
<xml_diff>
--- a/Guia_Ingles_Pronuncia.xlsx
+++ b/Guia_Ingles_Pronuncia.xlsx
@@ -2084,7 +2084,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4868,6 +4868,100 @@
       <c r="I59" s="2" t="inlineStr">
         <is>
           <t>Instagram @ingles.doimigrante (out/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>ISM</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Finais átonos</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>-ISM</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>i-zâm</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Falar "izãm" (vogal nasal) ou "is-mo" como em português. O final é átono e fecha no M, com os lábios fechados.</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>O S soa como Z. A tônica fica antes do sufixo: TUR-i-zâm, MÉ-kâ-ni-zâm.</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>The criticism of the tourism mechanism was fair.</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>Reel marco.essential (out/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>CIAN</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Sufixos com som de sh ou j</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>-CIAN</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>shân</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Falar "ci-ãn" separado ou "shãn" com vogal nasal.</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Mesma lógica do -TION e do -CIAL. A tônica cai na sílaba antes do sufixo: ték-NI-shân, i-lék-TRI-shân.</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>The technician called an electrician.</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>Reel marco.essential (out/2026)</t>
         </is>
       </c>
     </row>
@@ -4891,7 +4985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G469"/>
+  <dimension ref="A1:G476"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -20955,6 +21049,237 @@
         </is>
       </c>
       <c r="G469" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="2" t="inlineStr">
+        <is>
+          <t>ISM</t>
+        </is>
+      </c>
+      <c r="B470" s="2" t="n"/>
+      <c r="C470" s="2" t="inlineStr">
+        <is>
+          <t>tourism</t>
+        </is>
+      </c>
+      <c r="D470" s="2" t="inlineStr">
+        <is>
+          <t>TUR-i-zâm</t>
+        </is>
+      </c>
+      <c r="E470" s="2" t="inlineStr">
+        <is>
+          <t>ˈtʊrɪzəm</t>
+        </is>
+      </c>
+      <c r="F470" s="2" t="inlineStr">
+        <is>
+          <t>Reel marco.essential (out/2026)</t>
+        </is>
+      </c>
+      <c r="G470" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="2" t="inlineStr">
+        <is>
+          <t>ISM</t>
+        </is>
+      </c>
+      <c r="B471" s="2" t="n"/>
+      <c r="C471" s="2" t="inlineStr">
+        <is>
+          <t>mechanism</t>
+        </is>
+      </c>
+      <c r="D471" s="2" t="inlineStr">
+        <is>
+          <t>MÉ-kâ-ni-zâm</t>
+        </is>
+      </c>
+      <c r="E471" s="2" t="inlineStr">
+        <is>
+          <t>ˈmɛkənɪzəm</t>
+        </is>
+      </c>
+      <c r="F471" s="2" t="inlineStr">
+        <is>
+          <t>Reel marco.essential (out/2026)</t>
+        </is>
+      </c>
+      <c r="G471" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="2" t="inlineStr">
+        <is>
+          <t>ISM</t>
+        </is>
+      </c>
+      <c r="B472" s="2" t="n"/>
+      <c r="C472" s="2" t="inlineStr">
+        <is>
+          <t>criticism</t>
+        </is>
+      </c>
+      <c r="D472" s="2" t="inlineStr">
+        <is>
+          <t>KRI-ɾâ-si-zâm</t>
+        </is>
+      </c>
+      <c r="E472" s="2" t="inlineStr">
+        <is>
+          <t>ˈkrɪɾəsɪzəm</t>
+        </is>
+      </c>
+      <c r="F472" s="2" t="inlineStr">
+        <is>
+          <t>Reel marco.essential (out/2026)</t>
+        </is>
+      </c>
+      <c r="G472" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" s="2" t="inlineStr">
+        <is>
+          <t>CIAN</t>
+        </is>
+      </c>
+      <c r="B473" s="2" t="n"/>
+      <c r="C473" s="2" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+      <c r="D473" s="2" t="inlineStr">
+        <is>
+          <t>ték-NI-shân</t>
+        </is>
+      </c>
+      <c r="E473" s="2" t="inlineStr">
+        <is>
+          <t>tɛkˈnɪʃən</t>
+        </is>
+      </c>
+      <c r="F473" s="2" t="inlineStr">
+        <is>
+          <t>Reel marco.essential (out/2026)</t>
+        </is>
+      </c>
+      <c r="G473" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="2" t="inlineStr">
+        <is>
+          <t>CIAN</t>
+        </is>
+      </c>
+      <c r="B474" s="2" t="n"/>
+      <c r="C474" s="2" t="inlineStr">
+        <is>
+          <t>electrician</t>
+        </is>
+      </c>
+      <c r="D474" s="2" t="inlineStr">
+        <is>
+          <t>i-lék-TRI-shân</t>
+        </is>
+      </c>
+      <c r="E474" s="2" t="inlineStr">
+        <is>
+          <t>ɪlɛkˈtrɪʃən</t>
+        </is>
+      </c>
+      <c r="F474" s="2" t="inlineStr">
+        <is>
+          <t>Reel marco.essential (out/2026)</t>
+        </is>
+      </c>
+      <c r="G474" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" s="2" t="inlineStr">
+        <is>
+          <t>LE</t>
+        </is>
+      </c>
+      <c r="B475" s="2" t="n"/>
+      <c r="C475" s="2" t="inlineStr">
+        <is>
+          <t>bottle</t>
+        </is>
+      </c>
+      <c r="D475" s="2" t="inlineStr">
+        <is>
+          <t>BÁ-ɾâl</t>
+        </is>
+      </c>
+      <c r="E475" s="2" t="inlineStr">
+        <is>
+          <t>ˈbɑɾəl</t>
+        </is>
+      </c>
+      <c r="F475" s="2" t="inlineStr">
+        <is>
+          <t>Reel marco.essential (out/2026)</t>
+        </is>
+      </c>
+      <c r="G475" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="2" t="inlineStr">
+        <is>
+          <t>LE</t>
+        </is>
+      </c>
+      <c r="B476" s="2" t="n"/>
+      <c r="C476" s="2" t="inlineStr">
+        <is>
+          <t>settle</t>
+        </is>
+      </c>
+      <c r="D476" s="2" t="inlineStr">
+        <is>
+          <t>SÉ-ɾâl</t>
+        </is>
+      </c>
+      <c r="E476" s="2" t="inlineStr">
+        <is>
+          <t>ˈsɛɾəl</t>
+        </is>
+      </c>
+      <c r="F476" s="2" t="inlineStr">
+        <is>
+          <t>Reel marco.essential (out/2026)</t>
+        </is>
+      </c>
+      <c r="G476" s="2" t="inlineStr">
         <is>
           <t>treinar</t>
         </is>

</xml_diff>

<commit_message>
Guia: +5 palavras (took, umbrella, vitamin, selfie, apart) do vídeo @teachergiuliasartori sobre TAKE
took entra em OO (u curto); umbrella, vitamin, selfie e apart entram em GRAF.
Validação sem erros; IPA conferido no Cambridge US. PDF regenerado.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013eHjdS81LbDEqqSRnpMpTZ
</commit_message>
<xml_diff>
--- a/Guia_Ingles_Pronuncia.xlsx
+++ b/Guia_Ingles_Pronuncia.xlsx
@@ -4985,7 +4985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G476"/>
+  <dimension ref="A1:G481"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21280,6 +21280,175 @@
         </is>
       </c>
       <c r="G476" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="2" t="inlineStr">
+        <is>
+          <t>OO</t>
+        </is>
+      </c>
+      <c r="B477" s="2" t="inlineStr">
+        <is>
+          <t>u (curto)</t>
+        </is>
+      </c>
+      <c r="C477" s="2" t="inlineStr">
+        <is>
+          <t>took</t>
+        </is>
+      </c>
+      <c r="D477" s="2" t="inlineStr">
+        <is>
+          <t>TUK</t>
+        </is>
+      </c>
+      <c r="E477" s="2" t="inlineStr">
+        <is>
+          <t>tʊk</t>
+        </is>
+      </c>
+      <c r="F477" s="2" t="inlineStr">
+        <is>
+          <t>Vídeo @teachergiuliasartori sobre TAKE (out/2026)</t>
+        </is>
+      </c>
+      <c r="G477" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="2" t="inlineStr">
+        <is>
+          <t>GRAF</t>
+        </is>
+      </c>
+      <c r="B478" s="2" t="n"/>
+      <c r="C478" s="2" t="inlineStr">
+        <is>
+          <t>umbrella</t>
+        </is>
+      </c>
+      <c r="D478" s="2" t="inlineStr">
+        <is>
+          <t>âm-BRÉ-lâ</t>
+        </is>
+      </c>
+      <c r="E478" s="2" t="inlineStr">
+        <is>
+          <t>ʌmˈbrelə</t>
+        </is>
+      </c>
+      <c r="F478" s="2" t="inlineStr">
+        <is>
+          <t>Vídeo @teachergiuliasartori sobre TAKE (out/2026)</t>
+        </is>
+      </c>
+      <c r="G478" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" s="2" t="inlineStr">
+        <is>
+          <t>GRAF</t>
+        </is>
+      </c>
+      <c r="B479" s="2" t="n"/>
+      <c r="C479" s="2" t="inlineStr">
+        <is>
+          <t>vitamin</t>
+        </is>
+      </c>
+      <c r="D479" s="2" t="inlineStr">
+        <is>
+          <t>VÁI-ɾâ-min</t>
+        </is>
+      </c>
+      <c r="E479" s="2" t="inlineStr">
+        <is>
+          <t>ˈvaɪɾəmɪn</t>
+        </is>
+      </c>
+      <c r="F479" s="2" t="inlineStr">
+        <is>
+          <t>Vídeo @teachergiuliasartori sobre TAKE (out/2026)</t>
+        </is>
+      </c>
+      <c r="G479" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="2" t="inlineStr">
+        <is>
+          <t>GRAF</t>
+        </is>
+      </c>
+      <c r="B480" s="2" t="n"/>
+      <c r="C480" s="2" t="inlineStr">
+        <is>
+          <t>selfie</t>
+        </is>
+      </c>
+      <c r="D480" s="2" t="inlineStr">
+        <is>
+          <t>SÉL-fi</t>
+        </is>
+      </c>
+      <c r="E480" s="2" t="inlineStr">
+        <is>
+          <t>ˈselfi</t>
+        </is>
+      </c>
+      <c r="F480" s="2" t="inlineStr">
+        <is>
+          <t>Vídeo @teachergiuliasartori sobre TAKE (out/2026)</t>
+        </is>
+      </c>
+      <c r="G480" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" s="2" t="inlineStr">
+        <is>
+          <t>GRAF</t>
+        </is>
+      </c>
+      <c r="B481" s="2" t="n"/>
+      <c r="C481" s="2" t="inlineStr">
+        <is>
+          <t>apart</t>
+        </is>
+      </c>
+      <c r="D481" s="2" t="inlineStr">
+        <is>
+          <t>â-PÁRT</t>
+        </is>
+      </c>
+      <c r="E481" s="2" t="inlineStr">
+        <is>
+          <t>əˈpɑrt</t>
+        </is>
+      </c>
+      <c r="F481" s="2" t="inlineStr">
+        <is>
+          <t>Vídeo @teachergiuliasartori sobre TAKE (out/2026)</t>
+        </is>
+      </c>
+      <c r="G481" s="2" t="inlineStr">
         <is>
           <t>treinar</t>
         </is>

</xml_diff>

<commit_message>
Guia: grupo PHRASAL (tônica na partícula) com 7 phrasal verbs de take
take off/out/back/up/after/apart/down, do vídeo @teachergiuliasartori sobre TAKE.
Seção Tônica que muda. Validação sem erros; PDF regenerado.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013eHjdS81LbDEqqSRnpMpTZ
</commit_message>
<xml_diff>
--- a/Guia_Ingles_Pronuncia.xlsx
+++ b/Guia_Ingles_Pronuncia.xlsx
@@ -2084,7 +2084,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4962,6 +4962,53 @@
       <c r="I61" s="2" t="inlineStr">
         <is>
           <t>Reel marco.essential (out/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>PHRASAL</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Tônica que muda</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Phrasal verbs (verbo + partícula)</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>a tônica cai na partícula: take OFF, take OUT</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Acentuar o verbo e engolir a partícula: "TÊIK of", "TÊIK aut". Quem ouve entende só "take".</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Vale para a maioria dos phrasal verbs (turn ON, give UP, set UP). O substantivo composto volta a tônica para o verbo: o TAKEoff do avião × take OFF (decolar).</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Please take off the cover, take out the filter and take down the serial number.</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>Vídeo @teachergiuliasartori sobre TAKE (out/2026) + regra geral de tônica</t>
         </is>
       </c>
     </row>
@@ -4985,7 +5032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G481"/>
+  <dimension ref="A1:G488"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21449,6 +21496,265 @@
         </is>
       </c>
       <c r="G481" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" s="2" t="inlineStr">
+        <is>
+          <t>PHRASAL</t>
+        </is>
+      </c>
+      <c r="B482" s="2" t="inlineStr">
+        <is>
+          <t>take + partícula</t>
+        </is>
+      </c>
+      <c r="C482" s="2" t="inlineStr">
+        <is>
+          <t>take off</t>
+        </is>
+      </c>
+      <c r="D482" s="2" t="inlineStr">
+        <is>
+          <t>têik-ÁF</t>
+        </is>
+      </c>
+      <c r="E482" s="2" t="inlineStr">
+        <is>
+          <t>ˌteɪk ˈɑf</t>
+        </is>
+      </c>
+      <c r="F482" s="2" t="inlineStr">
+        <is>
+          <t>Vídeo @teachergiuliasartori sobre TAKE (out/2026)</t>
+        </is>
+      </c>
+      <c r="G482" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" s="2" t="inlineStr">
+        <is>
+          <t>PHRASAL</t>
+        </is>
+      </c>
+      <c r="B483" s="2" t="inlineStr">
+        <is>
+          <t>take + partícula</t>
+        </is>
+      </c>
+      <c r="C483" s="2" t="inlineStr">
+        <is>
+          <t>take out</t>
+        </is>
+      </c>
+      <c r="D483" s="2" t="inlineStr">
+        <is>
+          <t>têik-ÁUT</t>
+        </is>
+      </c>
+      <c r="E483" s="2" t="inlineStr">
+        <is>
+          <t>ˌteɪk ˈaʊt</t>
+        </is>
+      </c>
+      <c r="F483" s="2" t="inlineStr">
+        <is>
+          <t>Vídeo @teachergiuliasartori sobre TAKE (out/2026)</t>
+        </is>
+      </c>
+      <c r="G483" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" s="2" t="inlineStr">
+        <is>
+          <t>PHRASAL</t>
+        </is>
+      </c>
+      <c r="B484" s="2" t="inlineStr">
+        <is>
+          <t>take + partícula</t>
+        </is>
+      </c>
+      <c r="C484" s="2" t="inlineStr">
+        <is>
+          <t>take back</t>
+        </is>
+      </c>
+      <c r="D484" s="2" t="inlineStr">
+        <is>
+          <t>têik-BÆK</t>
+        </is>
+      </c>
+      <c r="E484" s="2" t="inlineStr">
+        <is>
+          <t>ˌteɪk ˈbæk</t>
+        </is>
+      </c>
+      <c r="F484" s="2" t="inlineStr">
+        <is>
+          <t>Vídeo @teachergiuliasartori sobre TAKE (out/2026)</t>
+        </is>
+      </c>
+      <c r="G484" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" s="2" t="inlineStr">
+        <is>
+          <t>PHRASAL</t>
+        </is>
+      </c>
+      <c r="B485" s="2" t="inlineStr">
+        <is>
+          <t>take + partícula</t>
+        </is>
+      </c>
+      <c r="C485" s="2" t="inlineStr">
+        <is>
+          <t>take up</t>
+        </is>
+      </c>
+      <c r="D485" s="2" t="inlineStr">
+        <is>
+          <t>têik-ÂP</t>
+        </is>
+      </c>
+      <c r="E485" s="2" t="inlineStr">
+        <is>
+          <t>ˌteɪk ˈʌp</t>
+        </is>
+      </c>
+      <c r="F485" s="2" t="inlineStr">
+        <is>
+          <t>Vídeo @teachergiuliasartori sobre TAKE (out/2026)</t>
+        </is>
+      </c>
+      <c r="G485" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" s="2" t="inlineStr">
+        <is>
+          <t>PHRASAL</t>
+        </is>
+      </c>
+      <c r="B486" s="2" t="inlineStr">
+        <is>
+          <t>take + partícula</t>
+        </is>
+      </c>
+      <c r="C486" s="2" t="inlineStr">
+        <is>
+          <t>take after</t>
+        </is>
+      </c>
+      <c r="D486" s="2" t="inlineStr">
+        <is>
+          <t>têik-ÆF-târ</t>
+        </is>
+      </c>
+      <c r="E486" s="2" t="inlineStr">
+        <is>
+          <t>ˌteɪk ˈæftɚ</t>
+        </is>
+      </c>
+      <c r="F486" s="2" t="inlineStr">
+        <is>
+          <t>Vídeo @teachergiuliasartori sobre TAKE (out/2026)</t>
+        </is>
+      </c>
+      <c r="G486" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" s="2" t="inlineStr">
+        <is>
+          <t>PHRASAL</t>
+        </is>
+      </c>
+      <c r="B487" s="2" t="inlineStr">
+        <is>
+          <t>take + partícula</t>
+        </is>
+      </c>
+      <c r="C487" s="2" t="inlineStr">
+        <is>
+          <t>take apart</t>
+        </is>
+      </c>
+      <c r="D487" s="2" t="inlineStr">
+        <is>
+          <t>têik â-PÁRT</t>
+        </is>
+      </c>
+      <c r="E487" s="2" t="inlineStr">
+        <is>
+          <t>ˌteɪk əˈpɑrt</t>
+        </is>
+      </c>
+      <c r="F487" s="2" t="inlineStr">
+        <is>
+          <t>Vídeo @teachergiuliasartori sobre TAKE (out/2026)</t>
+        </is>
+      </c>
+      <c r="G487" s="2" t="inlineStr">
+        <is>
+          <t>treinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" s="2" t="inlineStr">
+        <is>
+          <t>PHRASAL</t>
+        </is>
+      </c>
+      <c r="B488" s="2" t="inlineStr">
+        <is>
+          <t>take + partícula</t>
+        </is>
+      </c>
+      <c r="C488" s="2" t="inlineStr">
+        <is>
+          <t>take down</t>
+        </is>
+      </c>
+      <c r="D488" s="2" t="inlineStr">
+        <is>
+          <t>têik-DÁUN</t>
+        </is>
+      </c>
+      <c r="E488" s="2" t="inlineStr">
+        <is>
+          <t>ˌteɪk ˈdaʊn</t>
+        </is>
+      </c>
+      <c r="F488" s="2" t="inlineStr">
+        <is>
+          <t>Vídeo @teachergiuliasartori sobre TAKE (out/2026)</t>
+        </is>
+      </c>
+      <c r="G488" s="2" t="inlineStr">
         <is>
           <t>treinar</t>
         </is>

</xml_diff>